<commit_message>
Update Philly BYOB Restaurant_with_websites_merged_20251116.xlsx
</commit_message>
<xml_diff>
--- a/philly_yelp_crawler/data/Philly BYOB Restaurant_with_websites_merged_20251116.xlsx
+++ b/philly_yelp_crawler/data/Philly BYOB Restaurant_with_websites_merged_20251116.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\slow3\OneDrive\桌面\GitHubProjects\BYOB\philly_yelp_crawler\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27E673E6-2FE6-407D-982A-F616F4D9E32F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A94028BF-C3DE-405B-97C4-0B16EEE10570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="457">
   <si>
     <t>Name</t>
   </si>
@@ -1346,6 +1346,53 @@
   </si>
   <si>
     <t>https://www.umai-umai.com/</t>
+  </si>
+  <si>
+    <t>Chateau Rouge</t>
+  </si>
+  <si>
+    <t>2108 South St, Philadelphia, PA 19146</t>
+  </si>
+  <si>
+    <t>(445) 223-4110</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://chateaurougephilly.com/</t>
+  </si>
+  <si>
+    <t>https://www.yelp.com/biz/chateau-rouge-philadelphia</t>
+  </si>
+  <si>
+    <t>2025-11-17</t>
+  </si>
+  <si>
+    <t>Baby's Kusina + Market</t>
+  </si>
+  <si>
+    <t>2816 W Girard Ave, Philadelphia, PA 19130</t>
+  </si>
+  <si>
+    <t>https://babysphl.com/</t>
+  </si>
+  <si>
+    <t>https://www.yelp.com/biz/baby-s-kusina-market-philadelphia</t>
+  </si>
+  <si>
+    <t>Yuhiro Omakase Sushi</t>
+  </si>
+  <si>
+    <t>2146 E Susquehanna Ave, Philadelphia, PA 19125</t>
+  </si>
+  <si>
+    <t>(267) 876-7062</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://yuhirosushi.com/</t>
+  </si>
+  <si>
+    <t>https://www.yelp.com/biz/yuhiro-omakase-sushi-and-handroll-bar-philadelphia</t>
   </si>
 </sst>
 </file>
@@ -1717,7 +1764,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M68"/>
+  <dimension ref="A1:M71"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.5" customWidth="1"/>
@@ -4227,6 +4274,63 @@
         <v>285</v>
       </c>
     </row>
+    <row r="69" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>442</v>
+      </c>
+      <c r="B69" t="s">
+        <v>443</v>
+      </c>
+      <c r="C69" t="s">
+        <v>444</v>
+      </c>
+      <c r="D69" t="s">
+        <v>445</v>
+      </c>
+      <c r="E69" t="s">
+        <v>446</v>
+      </c>
+      <c r="M69" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="70" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>448</v>
+      </c>
+      <c r="B70" t="s">
+        <v>449</v>
+      </c>
+      <c r="D70" t="s">
+        <v>450</v>
+      </c>
+      <c r="E70" t="s">
+        <v>451</v>
+      </c>
+      <c r="M70" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="71" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>452</v>
+      </c>
+      <c r="B71" t="s">
+        <v>453</v>
+      </c>
+      <c r="C71" t="s">
+        <v>454</v>
+      </c>
+      <c r="D71" t="s">
+        <v>455</v>
+      </c>
+      <c r="E71" t="s">
+        <v>456</v>
+      </c>
+      <c r="M71" t="s">
+        <v>447</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>